<commit_message>
docs(tutorials)+samples: Lp2 = 2 ft buried on the reinforced slope; FEM-2 re-measured under the new verdict rules
The buried end of each geogrid sits under 4-16 ft of fill and grips
within about two feet, so Lp2 = 2 ft replaces the symmetric 4 ft on the
base workbook (LEM-8, LEM sample 9, FEM sample 1, FEM-2). FEM-2 is
re-measured at the new defaults: Spencer 1.587 unchanged, SSRM 1.543
elastic-perfectly-plastic and 1.481 peak-residual — identical from a
3,000 budget, so the budget section now teaches what the extension
rule does; no line is in pullout any more; the overburden law gets its
own short section. FEM-1's budget section and dialog shots follow the
new defaults.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/fem/files/xslope_reinforce_fem.xlsx
+++ b/docs/fem/files/xslope_reinforce_fem.xlsx
@@ -2595,7 +2595,7 @@
         <v>4.0</v>
       </c>
       <c r="L3" s="3">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="M3" s="3">
         <v>0.0</v>
@@ -2662,7 +2662,7 @@
         <v>4.0</v>
       </c>
       <c r="L4" s="3">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="M4" s="3">
         <v>0.0</v>
@@ -2723,7 +2723,7 @@
         <v>4.0</v>
       </c>
       <c r="L5" s="3">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="M5" s="3">
         <v>0.0</v>
@@ -2784,7 +2784,7 @@
         <v>4.0</v>
       </c>
       <c r="L6" s="3">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="M6" s="3">
         <v>0.0</v>
@@ -2842,7 +2842,7 @@
         <v>4.0</v>
       </c>
       <c r="L7" s="3">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="M7" s="3">
         <v>0.0</v>
@@ -2900,7 +2900,7 @@
         <v>4.0</v>
       </c>
       <c r="L8" s="3">
-        <v>4.0</v>
+        <v>2.0</v>
       </c>
       <c r="M8" s="3">
         <v>0.0</v>

</xml_diff>

<commit_message>
samples(reinforce): the published 4 ft/4 ft is restored; FEM-2 alone shortens the buried end
LEM sample 9 is xslope's transcription of the UTEXASED example and
develops over 4 ft at both ends again, as the example does; its note
states plain agreement. LEM-8 explains in one paragraph why a
practitioner would shorten the buried end or use Adhesion/Delta, and
that neither moves Spencer's 1.587 on this slope. FEM-2's builder
applies Lp2 = 2 ft itself and the page says what that changes (which
bar ends slip). FEM sample 1 re-locked at 1.509 under the current
engine with its companions regenerated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/fem/files/xslope_reinforce_fem.xlsx
+++ b/docs/fem/files/xslope_reinforce_fem.xlsx
@@ -2595,7 +2595,7 @@
         <v>4.0</v>
       </c>
       <c r="L3" s="3">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="M3" s="3">
         <v>0.0</v>
@@ -2662,7 +2662,7 @@
         <v>4.0</v>
       </c>
       <c r="L4" s="3">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="M4" s="3">
         <v>0.0</v>
@@ -2723,7 +2723,7 @@
         <v>4.0</v>
       </c>
       <c r="L5" s="3">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="M5" s="3">
         <v>0.0</v>
@@ -2784,7 +2784,7 @@
         <v>4.0</v>
       </c>
       <c r="L6" s="3">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="M6" s="3">
         <v>0.0</v>
@@ -2842,7 +2842,7 @@
         <v>4.0</v>
       </c>
       <c r="L7" s="3">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="M7" s="3">
         <v>0.0</v>
@@ -2900,7 +2900,7 @@
         <v>4.0</v>
       </c>
       <c r="L8" s="3">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="M8" s="3">
         <v>0.0</v>

</xml_diff>